<commit_message>
Stable version: absences + workdays reports with correct sorting and holidays
</commit_message>
<xml_diff>
--- a/data/output/absences_2026_02.xlsx
+++ b/data/output/absences_2026_02.xlsx
@@ -450,26 +450,26 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>036497310</t>
+          <t>047987630</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ΑΘΑΝΑΣΟΠΟΥΛΟΣ</t>
+          <t>ΣΤΑΜΑΤΟΠΟΥΛΟΣ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ΣΤΑΥΡΟΣ</t>
+          <t>ΝΙΚΟΛΑΟΣ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>09/02/2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -514,22 +514,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>037843072</t>
+          <t>036497310</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ΒΑΒΑΡΟΥΤΑ</t>
+          <t>ΑΘΑΝΑΣΟΠΟΥΛΟΣ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ΚΩΝΣΤΑΝΤΙΝΑ</t>
+          <t>ΣΤΑΥΡΟΣ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>037843072</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΒΑΒΑΡΟΥΤΑ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΚΩΝΣΤΑΝΤΙΝΑ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>11/02/2026</t>
+          <t>09/02/2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -574,12 +574,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>127063376</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΞΟΥΛΟΣ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -604,22 +604,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>141897793</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΔΙΔΑΧΟΥ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΑΦΡΟΔΙΤΗ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17/02/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -634,22 +634,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>141897793</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΔΙΔΑΧΟΥ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΑΦΡΟΔΙΤΗ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>18/02/2026</t>
+          <t>03/02/2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -664,22 +664,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>141897793</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΔΙΔΑΧΟΥ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΑΦΡΟΔΙΤΗ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19/02/2026</t>
+          <t>04/02/2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -694,22 +694,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>157133714</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΚΑΝΕΛΛΑΚΗΣ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΚΩΝΣΤΑΝΤΙΝΟΣ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>20/02/2026</t>
+          <t>02/02/2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -724,22 +724,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>157133714</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΣ</t>
+          <t>ΚΑΝΕΛΛΑΚΗΣ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΚΩΝΣΤΑΝΤΙΝΟΣ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>27/02/2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>170907466</t>
+          <t>160088100</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -764,12 +764,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ΓΕΩΡΓΙΟΣ</t>
+          <t>ΠΑΝΑΓΙΩΤΗΣ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>27/02/2026</t>
+          <t>11/02/2026</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>160088100</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ΠΑΝΑΓΙΩΤΗΣ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -844,22 +844,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>141897793</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΥ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ΑΦΡΟΔΙΤΗ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>17/02/2026</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -874,22 +874,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>141897793</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΥ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ΑΦΡΟΔΙΤΗ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>03/02/2026</t>
+          <t>18/02/2026</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -904,22 +904,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>141897793</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ΔΙΔΑΧΟΥ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ΑΦΡΟΔΙΤΗ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>04/02/2026</t>
+          <t>19/02/2026</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -934,22 +934,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>157133714</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ΚΑΝΕΛΛΑΚΗΣ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ΚΩΝΣΤΑΝΤΙΝΟΣ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>20/02/2026</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -964,22 +964,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>157133714</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ΚΑΝΕΛΛΑΚΗΣ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ΚΩΝΣΤΑΝΤΙΝΟΣ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>27/02/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>127063376</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ΞΟΥΛΟΣ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>02/02/2026</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1020,26 +1020,26 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>047987630</t>
+          <t>170907466</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ΣΤΑΜΑΤΟΠΟΥΛΟΣ</t>
+          <t>ΔΙΔΑΧΟΣ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ΝΙΚΟΛΑΟΣ</t>
+          <t>ΓΕΩΡΓΙΟΣ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>27/02/2026</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">

</xml_diff>